<commit_message>
feat: implement employee leave request system with dashboard views and localization support
</commit_message>
<xml_diff>
--- a/dummy_employees.xlsx
+++ b/dummy_employees.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\freelance\login system\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4A14FB2-868B-410D-8B45-3BB46B268DEB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{00DF324F-0F1F-46A9-A290-A436C792147B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -27,12 +27,6 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="181" uniqueCount="167">
   <si>
-    <t>Employee Name</t>
-  </si>
-  <si>
-    <t>Employee Name En</t>
-  </si>
-  <si>
     <t>Email Address</t>
   </si>
   <si>
@@ -526,6 +520,12 @@
   </si>
   <si>
     <t>2024-11-16</t>
+  </si>
+  <si>
+    <t>Employee Name (Arabic)</t>
+  </si>
+  <si>
+    <t>Employee Name (English)</t>
   </si>
 </sst>
 </file>
@@ -874,84 +874,84 @@
   <sheetData>
     <row r="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>165</v>
+      </c>
+      <c r="B1" t="s">
+        <v>166</v>
+      </c>
+      <c r="C1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="D1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="E1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="F1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="G1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="H1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="I1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="J1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="K1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="L1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="M1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="N1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="O1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="P1" t="s">
         <v>13</v>
-      </c>
-      <c r="O1" t="s">
-        <v>14</v>
-      </c>
-      <c r="P1" t="s">
-        <v>15</v>
       </c>
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C2" t="s">
         <v>16</v>
       </c>
-      <c r="B2" t="s">
+      <c r="D2" t="s">
         <v>17</v>
       </c>
-      <c r="C2" t="s">
+      <c r="E2" t="s">
         <v>18</v>
       </c>
-      <c r="D2" t="s">
+      <c r="F2" t="s">
         <v>19</v>
-      </c>
-      <c r="E2" t="s">
-        <v>20</v>
-      </c>
-      <c r="F2" t="s">
-        <v>21</v>
       </c>
       <c r="G2">
         <v>7264197415</v>
       </c>
       <c r="H2" t="s">
+        <v>20</v>
+      </c>
+      <c r="I2" t="s">
+        <v>21</v>
+      </c>
+      <c r="J2" t="s">
         <v>22</v>
-      </c>
-      <c r="I2" t="s">
-        <v>23</v>
-      </c>
-      <c r="J2" t="s">
-        <v>24</v>
       </c>
       <c r="K2">
         <v>5479</v>
@@ -966,42 +966,42 @@
         <v>168</v>
       </c>
       <c r="O2" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="P2" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>25</v>
+      </c>
+      <c r="B3" t="s">
+        <v>26</v>
+      </c>
+      <c r="C3" t="s">
         <v>27</v>
       </c>
-      <c r="B3" t="s">
+      <c r="D3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E3" t="s">
         <v>28</v>
       </c>
-      <c r="C3" t="s">
+      <c r="F3" t="s">
         <v>29</v>
-      </c>
-      <c r="D3" t="s">
-        <v>19</v>
-      </c>
-      <c r="E3" t="s">
-        <v>30</v>
-      </c>
-      <c r="F3" t="s">
-        <v>31</v>
       </c>
       <c r="G3">
         <v>5847755694</v>
       </c>
       <c r="H3" t="s">
+        <v>30</v>
+      </c>
+      <c r="I3" t="s">
+        <v>31</v>
+      </c>
+      <c r="J3" t="s">
         <v>32</v>
-      </c>
-      <c r="I3" t="s">
-        <v>33</v>
-      </c>
-      <c r="J3" t="s">
-        <v>34</v>
       </c>
       <c r="K3">
         <v>8205</v>
@@ -1016,42 +1016,42 @@
         <v>198</v>
       </c>
       <c r="O3" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="P3" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
+        <v>35</v>
+      </c>
+      <c r="B4" t="s">
+        <v>36</v>
+      </c>
+      <c r="C4" t="s">
         <v>37</v>
       </c>
-      <c r="B4" t="s">
+      <c r="D4" t="s">
+        <v>17</v>
+      </c>
+      <c r="E4" t="s">
         <v>38</v>
       </c>
-      <c r="C4" t="s">
+      <c r="F4" t="s">
         <v>39</v>
-      </c>
-      <c r="D4" t="s">
-        <v>19</v>
-      </c>
-      <c r="E4" t="s">
-        <v>40</v>
-      </c>
-      <c r="F4" t="s">
-        <v>41</v>
       </c>
       <c r="G4">
         <v>5897108289</v>
       </c>
       <c r="H4" t="s">
+        <v>40</v>
+      </c>
+      <c r="I4" t="s">
+        <v>41</v>
+      </c>
+      <c r="J4" t="s">
         <v>42</v>
-      </c>
-      <c r="I4" t="s">
-        <v>43</v>
-      </c>
-      <c r="J4" t="s">
-        <v>44</v>
       </c>
       <c r="K4">
         <v>9773</v>
@@ -1066,42 +1066,42 @@
         <v>499</v>
       </c>
       <c r="O4" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="P4" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
     </row>
     <row r="5" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
+        <v>45</v>
+      </c>
+      <c r="B5" t="s">
+        <v>46</v>
+      </c>
+      <c r="C5" t="s">
         <v>47</v>
       </c>
-      <c r="B5" t="s">
+      <c r="D5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E5" t="s">
         <v>48</v>
       </c>
-      <c r="C5" t="s">
+      <c r="F5" t="s">
         <v>49</v>
       </c>
-      <c r="D5" t="s">
-        <v>19</v>
-      </c>
-      <c r="E5" t="s">
+      <c r="G5" t="s">
         <v>50</v>
       </c>
-      <c r="F5" t="s">
+      <c r="H5" t="s">
         <v>51</v>
       </c>
-      <c r="G5" t="s">
+      <c r="I5" t="s">
         <v>52</v>
       </c>
-      <c r="H5" t="s">
+      <c r="J5" t="s">
         <v>53</v>
-      </c>
-      <c r="I5" t="s">
-        <v>54</v>
-      </c>
-      <c r="J5" t="s">
-        <v>55</v>
       </c>
       <c r="K5">
         <v>5382</v>
@@ -1116,42 +1116,42 @@
         <v>429</v>
       </c>
       <c r="O5" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="P5" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
     </row>
     <row r="6" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
+        <v>56</v>
+      </c>
+      <c r="B6" t="s">
+        <v>57</v>
+      </c>
+      <c r="C6" t="s">
         <v>58</v>
       </c>
-      <c r="B6" t="s">
+      <c r="D6" t="s">
+        <v>17</v>
+      </c>
+      <c r="E6" t="s">
         <v>59</v>
       </c>
-      <c r="C6" t="s">
+      <c r="F6" t="s">
         <v>60</v>
-      </c>
-      <c r="D6" t="s">
-        <v>19</v>
-      </c>
-      <c r="E6" t="s">
-        <v>61</v>
-      </c>
-      <c r="F6" t="s">
-        <v>62</v>
       </c>
       <c r="G6">
         <v>3028217636</v>
       </c>
       <c r="H6" t="s">
+        <v>61</v>
+      </c>
+      <c r="I6" t="s">
+        <v>62</v>
+      </c>
+      <c r="J6" t="s">
         <v>63</v>
-      </c>
-      <c r="I6" t="s">
-        <v>64</v>
-      </c>
-      <c r="J6" t="s">
-        <v>65</v>
       </c>
       <c r="K6">
         <v>3192</v>
@@ -1166,42 +1166,42 @@
         <v>430</v>
       </c>
       <c r="O6" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="P6" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
     </row>
     <row r="7" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
+        <v>66</v>
+      </c>
+      <c r="B7" t="s">
+        <v>67</v>
+      </c>
+      <c r="C7" t="s">
         <v>68</v>
       </c>
-      <c r="B7" t="s">
+      <c r="D7" t="s">
+        <v>17</v>
+      </c>
+      <c r="E7" t="s">
         <v>69</v>
       </c>
-      <c r="C7" t="s">
+      <c r="F7" t="s">
         <v>70</v>
-      </c>
-      <c r="D7" t="s">
-        <v>19</v>
-      </c>
-      <c r="E7" t="s">
-        <v>71</v>
-      </c>
-      <c r="F7" t="s">
-        <v>72</v>
       </c>
       <c r="G7">
         <v>7585943456</v>
       </c>
       <c r="H7" t="s">
+        <v>71</v>
+      </c>
+      <c r="I7" t="s">
+        <v>72</v>
+      </c>
+      <c r="J7" t="s">
         <v>73</v>
-      </c>
-      <c r="I7" t="s">
-        <v>74</v>
-      </c>
-      <c r="J7" t="s">
-        <v>75</v>
       </c>
       <c r="K7">
         <v>5396</v>
@@ -1216,42 +1216,42 @@
         <v>198</v>
       </c>
       <c r="O7" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="P7" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="8" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
+        <v>76</v>
+      </c>
+      <c r="B8" t="s">
+        <v>77</v>
+      </c>
+      <c r="C8" t="s">
         <v>78</v>
       </c>
-      <c r="B8" t="s">
+      <c r="D8" t="s">
+        <v>17</v>
+      </c>
+      <c r="E8" t="s">
         <v>79</v>
       </c>
-      <c r="C8" t="s">
+      <c r="F8" t="s">
         <v>80</v>
-      </c>
-      <c r="D8" t="s">
-        <v>19</v>
-      </c>
-      <c r="E8" t="s">
-        <v>81</v>
-      </c>
-      <c r="F8" t="s">
-        <v>82</v>
       </c>
       <c r="G8">
         <v>8050933996</v>
       </c>
       <c r="H8" t="s">
+        <v>81</v>
+      </c>
+      <c r="I8" t="s">
+        <v>82</v>
+      </c>
+      <c r="J8" t="s">
         <v>83</v>
-      </c>
-      <c r="I8" t="s">
-        <v>84</v>
-      </c>
-      <c r="J8" t="s">
-        <v>85</v>
       </c>
       <c r="K8">
         <v>9801</v>
@@ -1266,42 +1266,42 @@
         <v>249</v>
       </c>
       <c r="O8" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="P8" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
     </row>
     <row r="9" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
+        <v>86</v>
+      </c>
+      <c r="B9" t="s">
+        <v>87</v>
+      </c>
+      <c r="C9" t="s">
         <v>88</v>
       </c>
-      <c r="B9" t="s">
+      <c r="D9" t="s">
+        <v>17</v>
+      </c>
+      <c r="E9" t="s">
         <v>89</v>
       </c>
-      <c r="C9" t="s">
+      <c r="F9" t="s">
         <v>90</v>
-      </c>
-      <c r="D9" t="s">
-        <v>19</v>
-      </c>
-      <c r="E9" t="s">
-        <v>91</v>
-      </c>
-      <c r="F9" t="s">
-        <v>92</v>
       </c>
       <c r="G9">
         <v>4231958416</v>
       </c>
       <c r="H9" t="s">
+        <v>91</v>
+      </c>
+      <c r="I9" t="s">
+        <v>92</v>
+      </c>
+      <c r="J9" t="s">
         <v>93</v>
-      </c>
-      <c r="I9" t="s">
-        <v>94</v>
-      </c>
-      <c r="J9" t="s">
-        <v>95</v>
       </c>
       <c r="K9">
         <v>7875</v>
@@ -1316,42 +1316,42 @@
         <v>353</v>
       </c>
       <c r="O9" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="P9" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
     </row>
     <row r="10" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
+        <v>96</v>
+      </c>
+      <c r="B10" t="s">
+        <v>97</v>
+      </c>
+      <c r="C10" t="s">
         <v>98</v>
       </c>
-      <c r="B10" t="s">
+      <c r="D10" t="s">
+        <v>17</v>
+      </c>
+      <c r="E10" t="s">
         <v>99</v>
       </c>
-      <c r="C10" t="s">
+      <c r="F10" t="s">
         <v>100</v>
-      </c>
-      <c r="D10" t="s">
-        <v>19</v>
-      </c>
-      <c r="E10" t="s">
-        <v>101</v>
-      </c>
-      <c r="F10" t="s">
-        <v>102</v>
       </c>
       <c r="G10">
         <v>2091054768</v>
       </c>
       <c r="H10" t="s">
+        <v>101</v>
+      </c>
+      <c r="I10" t="s">
+        <v>102</v>
+      </c>
+      <c r="J10" t="s">
         <v>103</v>
-      </c>
-      <c r="I10" t="s">
-        <v>104</v>
-      </c>
-      <c r="J10" t="s">
-        <v>105</v>
       </c>
       <c r="K10">
         <v>8053</v>
@@ -1366,42 +1366,42 @@
         <v>237</v>
       </c>
       <c r="O10" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="P10" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
     </row>
     <row r="11" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
+        <v>106</v>
+      </c>
+      <c r="B11" t="s">
+        <v>107</v>
+      </c>
+      <c r="C11" t="s">
         <v>108</v>
       </c>
-      <c r="B11" t="s">
+      <c r="D11" t="s">
+        <v>17</v>
+      </c>
+      <c r="E11" t="s">
         <v>109</v>
       </c>
-      <c r="C11" t="s">
+      <c r="F11" t="s">
         <v>110</v>
-      </c>
-      <c r="D11" t="s">
-        <v>19</v>
-      </c>
-      <c r="E11" t="s">
-        <v>111</v>
-      </c>
-      <c r="F11" t="s">
-        <v>112</v>
       </c>
       <c r="G11">
         <v>4158466052</v>
       </c>
       <c r="H11" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="I11">
         <v>16895788153</v>
       </c>
       <c r="J11" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="K11">
         <v>4068</v>
@@ -1416,42 +1416,42 @@
         <v>399</v>
       </c>
       <c r="O11" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="P11" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
     </row>
     <row r="12" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
+        <v>115</v>
+      </c>
+      <c r="B12" t="s">
+        <v>116</v>
+      </c>
+      <c r="C12" t="s">
         <v>117</v>
       </c>
-      <c r="B12" t="s">
+      <c r="D12" t="s">
+        <v>17</v>
+      </c>
+      <c r="E12" t="s">
         <v>118</v>
       </c>
-      <c r="C12" t="s">
+      <c r="F12" t="s">
         <v>119</v>
-      </c>
-      <c r="D12" t="s">
-        <v>19</v>
-      </c>
-      <c r="E12" t="s">
-        <v>120</v>
-      </c>
-      <c r="F12" t="s">
-        <v>121</v>
       </c>
       <c r="G12">
         <v>5065284809</v>
       </c>
       <c r="H12" t="s">
+        <v>120</v>
+      </c>
+      <c r="I12" t="s">
+        <v>121</v>
+      </c>
+      <c r="J12" t="s">
         <v>122</v>
-      </c>
-      <c r="I12" t="s">
-        <v>123</v>
-      </c>
-      <c r="J12" t="s">
-        <v>124</v>
       </c>
       <c r="K12">
         <v>3554</v>
@@ -1466,42 +1466,42 @@
         <v>18</v>
       </c>
       <c r="O12" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="P12" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
     </row>
     <row r="13" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
+        <v>125</v>
+      </c>
+      <c r="B13" t="s">
+        <v>126</v>
+      </c>
+      <c r="C13" t="s">
         <v>127</v>
       </c>
-      <c r="B13" t="s">
+      <c r="D13" t="s">
+        <v>17</v>
+      </c>
+      <c r="E13" t="s">
         <v>128</v>
       </c>
-      <c r="C13" t="s">
+      <c r="F13" t="s">
         <v>129</v>
-      </c>
-      <c r="D13" t="s">
-        <v>19</v>
-      </c>
-      <c r="E13" t="s">
-        <v>130</v>
-      </c>
-      <c r="F13" t="s">
-        <v>131</v>
       </c>
       <c r="G13">
         <v>5257436678</v>
       </c>
       <c r="H13" t="s">
+        <v>130</v>
+      </c>
+      <c r="I13" t="s">
+        <v>131</v>
+      </c>
+      <c r="J13" t="s">
         <v>132</v>
-      </c>
-      <c r="I13" t="s">
-        <v>133</v>
-      </c>
-      <c r="J13" t="s">
-        <v>134</v>
       </c>
       <c r="K13">
         <v>9598</v>
@@ -1516,42 +1516,42 @@
         <v>305</v>
       </c>
       <c r="O13" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="P13" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
     </row>
     <row r="14" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
+        <v>135</v>
+      </c>
+      <c r="B14" t="s">
+        <v>136</v>
+      </c>
+      <c r="C14" t="s">
         <v>137</v>
       </c>
-      <c r="B14" t="s">
+      <c r="D14" t="s">
+        <v>17</v>
+      </c>
+      <c r="E14" t="s">
         <v>138</v>
       </c>
-      <c r="C14" t="s">
+      <c r="F14" t="s">
         <v>139</v>
-      </c>
-      <c r="D14" t="s">
-        <v>19</v>
-      </c>
-      <c r="E14" t="s">
-        <v>140</v>
-      </c>
-      <c r="F14" t="s">
-        <v>141</v>
       </c>
       <c r="G14">
         <v>7860728098</v>
       </c>
       <c r="H14" t="s">
+        <v>140</v>
+      </c>
+      <c r="I14" t="s">
+        <v>141</v>
+      </c>
+      <c r="J14" t="s">
         <v>142</v>
-      </c>
-      <c r="I14" t="s">
-        <v>143</v>
-      </c>
-      <c r="J14" t="s">
-        <v>144</v>
       </c>
       <c r="K14">
         <v>6734</v>
@@ -1566,42 +1566,42 @@
         <v>133</v>
       </c>
       <c r="O14" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="P14" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
     </row>
     <row r="15" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
+        <v>145</v>
+      </c>
+      <c r="B15" t="s">
+        <v>146</v>
+      </c>
+      <c r="C15" t="s">
         <v>147</v>
       </c>
-      <c r="B15" t="s">
+      <c r="D15" t="s">
+        <v>17</v>
+      </c>
+      <c r="E15" t="s">
         <v>148</v>
       </c>
-      <c r="C15" t="s">
+      <c r="F15" t="s">
         <v>149</v>
-      </c>
-      <c r="D15" t="s">
-        <v>19</v>
-      </c>
-      <c r="E15" t="s">
-        <v>150</v>
-      </c>
-      <c r="F15" t="s">
-        <v>151</v>
       </c>
       <c r="G15">
         <v>7317095106</v>
       </c>
       <c r="H15" t="s">
+        <v>150</v>
+      </c>
+      <c r="I15" t="s">
+        <v>151</v>
+      </c>
+      <c r="J15" t="s">
         <v>152</v>
-      </c>
-      <c r="I15" t="s">
-        <v>153</v>
-      </c>
-      <c r="J15" t="s">
-        <v>154</v>
       </c>
       <c r="K15">
         <v>5092</v>
@@ -1616,42 +1616,42 @@
         <v>236</v>
       </c>
       <c r="O15" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="P15" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
     </row>
     <row r="16" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
+        <v>155</v>
+      </c>
+      <c r="B16" t="s">
+        <v>156</v>
+      </c>
+      <c r="C16" t="s">
         <v>157</v>
       </c>
-      <c r="B16" t="s">
+      <c r="D16" t="s">
+        <v>17</v>
+      </c>
+      <c r="E16" t="s">
         <v>158</v>
       </c>
-      <c r="C16" t="s">
+      <c r="F16" t="s">
         <v>159</v>
-      </c>
-      <c r="D16" t="s">
-        <v>19</v>
-      </c>
-      <c r="E16" t="s">
-        <v>160</v>
-      </c>
-      <c r="F16" t="s">
-        <v>161</v>
       </c>
       <c r="G16">
         <v>2984528123</v>
       </c>
       <c r="H16" t="s">
+        <v>160</v>
+      </c>
+      <c r="I16" t="s">
+        <v>161</v>
+      </c>
+      <c r="J16" t="s">
         <v>162</v>
-      </c>
-      <c r="I16" t="s">
-        <v>163</v>
-      </c>
-      <c r="J16" t="s">
-        <v>164</v>
       </c>
       <c r="K16">
         <v>4541</v>
@@ -1666,10 +1666,10 @@
         <v>257</v>
       </c>
       <c r="O16" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="P16" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: implement EmployeeService for CRUD operations and add localization and views for employee management modules
</commit_message>
<xml_diff>
--- a/dummy_employees.xlsx
+++ b/dummy_employees.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\freelance\login system\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{00DF324F-0F1F-46A9-A290-A436C792147B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{51E516C4-45D8-413C-847D-42413869FBE6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -532,10 +532,16 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
       <name val="Calibri"/>
     </font>
   </fonts>
@@ -556,13 +562,16 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -1079,7 +1088,7 @@
       <c r="B5" t="s">
         <v>46</v>
       </c>
-      <c r="C5" t="s">
+      <c r="C5" s="1" t="s">
         <v>47</v>
       </c>
       <c r="D5" t="s">
@@ -1279,7 +1288,7 @@
       <c r="B9" t="s">
         <v>87</v>
       </c>
-      <c r="C9" t="s">
+      <c r="C9" s="1" t="s">
         <v>88</v>
       </c>
       <c r="D9" t="s">
@@ -1673,6 +1682,10 @@
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="C9" r:id="rId1" xr:uid="{31B62BBD-5730-4F0C-BCBB-50DAD709F9E9}"/>
+    <hyperlink ref="C5" r:id="rId2" xr:uid="{D1D31779-3072-427C-A4A9-F5B920DF6C7C}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: implement asset management controller and enhance payroll system with allowance tracking and backfill support
</commit_message>
<xml_diff>
--- a/dummy_employees.xlsx
+++ b/dummy_employees.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\freelance\login system\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{51E516C4-45D8-413C-847D-42413869FBE6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A4AF64D-5949-45F5-92F8-DC0F7A63095E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -879,6 +879,10 @@
   <cols>
     <col min="1" max="1" width="23.140625" customWidth="1"/>
     <col min="2" max="2" width="30.140625" customWidth="1"/>
+    <col min="11" max="11" width="18.28515625" customWidth="1"/>
+    <col min="12" max="12" width="15.42578125" customWidth="1"/>
+    <col min="13" max="13" width="17.140625" customWidth="1"/>
+    <col min="14" max="14" width="22.85546875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:16" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
feat: implement client management module with detailed views and localized UI components
</commit_message>
<xml_diff>
--- a/dummy_employees.xlsx
+++ b/dummy_employees.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\freelance\login system\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C2543E2-0010-48FE-A65C-11213238C2AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{230481A2-62E1-4952-9876-AD210FFFF97D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1642,7 +1642,7 @@
       <c r="B16" t="s">
         <v>156</v>
       </c>
-      <c r="C16" t="s">
+      <c r="C16" s="1" t="s">
         <v>157</v>
       </c>
       <c r="D16" t="s">
@@ -1689,6 +1689,7 @@
   <hyperlinks>
     <hyperlink ref="C9" r:id="rId1" xr:uid="{31B62BBD-5730-4F0C-BCBB-50DAD709F9E9}"/>
     <hyperlink ref="C5" r:id="rId2" xr:uid="{D1D31779-3072-427C-A4A9-F5B920DF6C7C}"/>
+    <hyperlink ref="C16" r:id="rId3" xr:uid="{004F3C4E-EEB7-4028-A58C-9F39C65D6BD1}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>